<commit_message>
update predictors excel and eda notebook
</commit_message>
<xml_diff>
--- a/02_eda/predictors.xlsx
+++ b/02_eda/predictors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/samswitz/GitHub/STAT-431-Final-Project/02_eda/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3666C05C-02FD-A249-8134-B6FDE8B40F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{517DABFD-FBC3-174A-BFC4-7823B2363496}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -625,9 +625,6 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" t="b">
-        <v>1</v>
-      </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -739,9 +736,6 @@
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>33</v>
-      </c>
-      <c r="B34" t="b">
-        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">

</xml_diff>